<commit_message>
feat: implement chat UI components, backend routes, and scheduler integration for marketing tool functionality
</commit_message>
<xml_diff>
--- a/frontend/src/assets/scheduler_template.xlsx
+++ b/frontend/src/assets/scheduler_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sharm\Documents\tool_v1\marketing_tool - v1\frontend\src\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8193DCFD-DEB9-42C1-92FB-BD20A4468450}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD039D10-ECE8-44D0-901A-15974D1C0BF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -86,7 +86,7 @@
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    Scheduled date and time for publishing or sending the content.  Enter time in UTC</t>
+    Scheduled date and time for publishing or sending the content.  Format 2026-08-20 11:20:00+05:30</t>
       </text>
     </comment>
   </commentList>
@@ -94,7 +94,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>post_type</t>
   </si>
@@ -115,6 +115,9 @@
   </si>
   <si>
     <t>scheduled_time</t>
+  </si>
+  <si>
+    <t>2026-08-20 11:20:00+05:30</t>
   </si>
 </sst>
 </file>
@@ -570,7 +573,7 @@
 </text>
   </threadedComment>
   <threadedComment ref="G1" dT="2026-08-14T05:33:37.60" personId="{8774E626-41FE-412B-95BB-B03DD1ACAA15}" id="{2F9431F2-770A-448D-8795-C304912ACB5C}">
-    <text>Scheduled date and time for publishing or sending the content.  Enter time in UTC</text>
+    <text>Scheduled date and time for publishing or sending the content.  Format 2026-08-20 11:20:00+05:30</text>
   </threadedComment>
 </ThreadedComments>
 </file>
@@ -616,6 +619,9 @@
       <c r="C2" s="3"/>
       <c r="D2"/>
       <c r="E2"/>
+      <c r="G2" s="2" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="3" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C3" s="3"/>

</xml_diff>